<commit_message>
Make weighted enrollment calculations use dynamic formulas across multiple workbook types
Update excel export logic to import and utilize the setFormula helper function, allowing weighted enrollment populations (SPED, ELL, Economically Disadvantaged) to be dynamically calculated using formulas in the Underwriting, Lender Pro Forma, and Standard Export workbooks. This ensures that changes to assumption values in Excel automatically update downstream totals and percentages.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 46f5b3d4-fee0-435d-bdc9-71834e4913d6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/1ucI1Ab
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Homeschool_Co-Op_Mixed.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Homeschool_Co-Op_Mixed.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="220">
   <si>
     <t>How to Use This Workbook</t>
   </si>
@@ -310,52 +310,40 @@
     <t>WEIGHTED ENROLLMENT POPULATIONS</t>
   </si>
   <si>
+    <t>Population</t>
+  </si>
+  <si>
+    <t>Year 1</t>
+  </si>
+  <si>
+    <t>Year 2</t>
+  </si>
+  <si>
+    <t>Year 3</t>
+  </si>
+  <si>
+    <t>Year 4</t>
+  </si>
+  <si>
+    <t>Year 5</t>
+  </si>
+  <si>
     <t>Special Education (SPED)</t>
   </si>
   <si>
-    <t>3  /  4  /  5  /  6  /  6</t>
-  </si>
-  <si>
     <t>English Language Learners (ELL)</t>
   </si>
   <si>
-    <t>2  /  3  /  4  /  5  /  5</t>
-  </si>
-  <si>
     <t>Economically Disadvantaged</t>
   </si>
   <si>
-    <t>5  /  7  /  9  /  10  /  12</t>
-  </si>
-  <si>
     <t>Total Weighted Students</t>
   </si>
   <si>
-    <t>10  /  14  /  18  /  21  /  23</t>
-  </si>
-  <si>
     <t>Weighted % of Enrollment</t>
   </si>
   <si>
-    <t>67%  /  64%  /  60%  /  58%  /  57%</t>
-  </si>
-  <si>
     <t>Revenue &amp; Expense Drivers</t>
-  </si>
-  <si>
-    <t>Year 1</t>
-  </si>
-  <si>
-    <t>Year 2</t>
-  </si>
-  <si>
-    <t>Year 3</t>
-  </si>
-  <si>
-    <t>Year 4</t>
-  </si>
-  <si>
-    <t>Year 5</t>
   </si>
   <si>
     <t>Enrollment</t>
@@ -953,7 +941,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -987,11 +975,18 @@
     <xf numFmtId="166" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1789,7 +1784,7 @@
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1810,528 +1805,528 @@
       <c r="H3" s="12"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="48" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4" s="49" t="s">
+        <v>171</v>
+      </c>
+      <c r="F4" s="50" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="51" t="s">
+        <v>173</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="52" t="s">
+        <v>99</v>
+      </c>
+      <c r="F6" s="52" t="s">
+        <v>100</v>
+      </c>
+      <c r="G6" s="52" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="D4" s="48" t="s">
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="32">
+        <v>15</v>
+      </c>
+      <c r="D7" s="32">
+        <v>22</v>
+      </c>
+      <c r="E7" s="32">
+        <v>30</v>
+      </c>
+      <c r="F7" s="32">
+        <v>36</v>
+      </c>
+      <c r="G7" s="32">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="F4" s="49" t="s">
+      <c r="C8" s="33">
+        <v>108000</v>
+      </c>
+      <c r="D8" s="33">
+        <v>161620</v>
+      </c>
+      <c r="E8" s="33">
+        <v>225789</v>
+      </c>
+      <c r="F8" s="33">
+        <v>278367.204</v>
+      </c>
+      <c r="G8" s="33">
+        <v>318142.46680000005</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="31" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="6" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="50" t="s">
+      <c r="C9" s="33">
+        <v>93600</v>
+      </c>
+      <c r="D9" s="33">
+        <v>96408</v>
+      </c>
+      <c r="E9" s="33">
+        <v>99300.23999999999</v>
+      </c>
+      <c r="F9" s="33">
+        <v>141617.4192</v>
+      </c>
+      <c r="G9" s="33">
+        <v>145865.94177600002</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="C6" s="51" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" s="51" t="s">
-        <v>108</v>
-      </c>
-      <c r="E6" s="51" t="s">
-        <v>109</v>
-      </c>
-      <c r="F6" s="51" t="s">
-        <v>110</v>
-      </c>
-      <c r="G6" s="51" t="s">
-        <v>111</v>
-      </c>
-      <c r="H6" s="51" t="s">
+      <c r="C10" s="33">
+        <v>35550</v>
+      </c>
+      <c r="D10" s="33">
+        <v>45522.86666666667</v>
+      </c>
+      <c r="E10" s="33">
+        <v>63304.53602635659</v>
+      </c>
+      <c r="F10" s="33">
+        <v>90773.3936127556</v>
+      </c>
+      <c r="G10" s="33">
+        <v>131957.43501823914</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="31" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7" s="31">
-        <v>15</v>
-      </c>
-      <c r="D7" s="31">
-        <v>22</v>
-      </c>
-      <c r="E7" s="31">
-        <v>30</v>
-      </c>
-      <c r="F7" s="31">
-        <v>36</v>
-      </c>
-      <c r="G7" s="31">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
+      <c r="C11" s="33">
+        <v>0</v>
+      </c>
+      <c r="D11" s="33">
+        <v>0</v>
+      </c>
+      <c r="E11" s="33">
+        <v>0</v>
+      </c>
+      <c r="F11" s="33">
+        <v>0</v>
+      </c>
+      <c r="G11" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="34" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" s="36">
+        <v>-21150</v>
+      </c>
+      <c r="D12" s="37">
+        <v>19689.13333333333</v>
+      </c>
+      <c r="E12" s="37">
+        <v>63184.22397364341</v>
+      </c>
+      <c r="F12" s="37">
+        <v>45976.391187244444</v>
+      </c>
+      <c r="G12" s="37">
+        <v>40319.090005760896</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="36">
+        <v>-21150</v>
+      </c>
+      <c r="D13" s="36">
+        <v>-1460.8666666666686</v>
+      </c>
+      <c r="E13" s="37">
+        <v>61723.357306976744</v>
+      </c>
+      <c r="F13" s="37">
+        <v>107699.74849422119</v>
+      </c>
+      <c r="G13" s="37">
+        <v>148018.83849998208</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" s="53">
+        <v>-0.19583333333333333</v>
+      </c>
+      <c r="D14" s="54">
+        <v>0.12182361918904425</v>
+      </c>
+      <c r="E14" s="54">
+        <v>0.27983747646538765</v>
+      </c>
+      <c r="F14" s="54">
+        <v>0.16516453995508912</v>
+      </c>
+      <c r="G14" s="54">
+        <v>0.12673281379661727</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="C8" s="32">
-        <v>108000</v>
-      </c>
-      <c r="D8" s="32">
-        <v>161620</v>
-      </c>
-      <c r="E8" s="32">
-        <v>225789</v>
-      </c>
-      <c r="F8" s="32">
-        <v>278367.204</v>
-      </c>
-      <c r="G8" s="32">
-        <v>318142.46680000005</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="30" t="s">
+      <c r="C15" s="55">
+        <v>7200</v>
+      </c>
+      <c r="D15" s="55">
+        <v>7346.363636363636</v>
+      </c>
+      <c r="E15" s="55">
+        <v>7526.3</v>
+      </c>
+      <c r="F15" s="55">
+        <v>7732.422333333334</v>
+      </c>
+      <c r="G15" s="55">
+        <v>7953.561670000001</v>
+      </c>
+      <c r="H15" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="C9" s="32">
-        <v>93600</v>
-      </c>
-      <c r="D9" s="32">
-        <v>96408</v>
-      </c>
-      <c r="E9" s="32">
-        <v>99300.23999999999</v>
-      </c>
-      <c r="F9" s="32">
-        <v>141617.4192</v>
-      </c>
-      <c r="G9" s="32">
-        <v>145865.94177600002</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="30" t="s">
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="C10" s="32">
-        <v>35550</v>
-      </c>
-      <c r="D10" s="32">
-        <v>45522.86666666667</v>
-      </c>
-      <c r="E10" s="32">
-        <v>63304.53602635659</v>
-      </c>
-      <c r="F10" s="32">
-        <v>90773.3936127556</v>
-      </c>
-      <c r="G10" s="32">
-        <v>131957.43501823914</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="30" t="s">
+      <c r="C16" s="53">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="D16" s="57">
+        <v>0.5965103328795941</v>
+      </c>
+      <c r="E16" s="54">
+        <v>0.439792195368242</v>
+      </c>
+      <c r="F16" s="54">
+        <v>0.5087431894455497</v>
+      </c>
+      <c r="G16" s="54">
+        <v>0.4584925214265674</v>
+      </c>
+      <c r="H16" s="56" t="s">
         <v>182</v>
       </c>
-      <c r="C11" s="32">
-        <v>0</v>
-      </c>
-      <c r="D11" s="32">
-        <v>0</v>
-      </c>
-      <c r="E11" s="32">
-        <v>0</v>
-      </c>
-      <c r="F11" s="32">
-        <v>0</v>
-      </c>
-      <c r="G11" s="32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="33" t="s">
-        <v>137</v>
-      </c>
-      <c r="C12" s="35">
-        <v>-21150</v>
-      </c>
-      <c r="D12" s="36">
-        <v>19689.13333333333</v>
-      </c>
-      <c r="E12" s="36">
-        <v>63184.22397364341</v>
-      </c>
-      <c r="F12" s="36">
-        <v>45976.391187244444</v>
-      </c>
-      <c r="G12" s="36">
-        <v>40319.090005760896</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="35">
-        <v>-21150</v>
-      </c>
-      <c r="D13" s="35">
-        <v>-1460.8666666666686</v>
-      </c>
-      <c r="E13" s="36">
-        <v>61723.357306976744</v>
-      </c>
-      <c r="F13" s="36">
-        <v>107699.74849422119</v>
-      </c>
-      <c r="G13" s="36">
-        <v>148018.83849998208</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="33" t="s">
-        <v>138</v>
-      </c>
-      <c r="C14" s="52">
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="34" t="s">
+        <v>183</v>
+      </c>
+      <c r="C17" s="53">
+        <v>0.2388888888888889</v>
+      </c>
+      <c r="D17" s="57">
+        <v>0.16429278554634325</v>
+      </c>
+      <c r="E17" s="54">
+        <v>0.12103325269620419</v>
+      </c>
+      <c r="F17" s="54">
+        <v>0.10103766643260505</v>
+      </c>
+      <c r="G17" s="54">
+        <v>0.09098580037985765</v>
+      </c>
+      <c r="H17" s="56" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="53">
         <v>-0.19583333333333333</v>
       </c>
-      <c r="D14" s="53">
+      <c r="D18" s="54">
         <v>0.12182361918904425</v>
       </c>
-      <c r="E14" s="53">
-        <v>0.27983747646538765</v>
-      </c>
-      <c r="F14" s="53">
-        <v>0.16516453995508912</v>
-      </c>
-      <c r="G14" s="53">
+      <c r="E18" s="54">
+        <v>0.2798374764653877</v>
+      </c>
+      <c r="F18" s="54">
+        <v>0.16516453995508906</v>
+      </c>
+      <c r="G18" s="54">
         <v>0.12673281379661727</v>
       </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="33" t="s">
-        <v>183</v>
-      </c>
-      <c r="C15" s="54">
-        <v>7200</v>
-      </c>
-      <c r="D15" s="54">
-        <v>7346.363636363636</v>
-      </c>
-      <c r="E15" s="54">
-        <v>7526.3</v>
-      </c>
-      <c r="F15" s="54">
-        <v>7732.422333333334</v>
-      </c>
-      <c r="G15" s="54">
-        <v>7953.561670000001</v>
-      </c>
-      <c r="H15" s="55" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="33" t="s">
+      <c r="H18" s="56" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="52">
-        <v>0.8666666666666667</v>
-      </c>
-      <c r="D16" s="56">
-        <v>0.5965103328795941</v>
-      </c>
-      <c r="E16" s="53">
-        <v>0.439792195368242</v>
-      </c>
-      <c r="F16" s="53">
-        <v>0.5087431894455497</v>
-      </c>
-      <c r="G16" s="53">
-        <v>0.4584925214265674</v>
-      </c>
-      <c r="H16" s="55" t="s">
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="34" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="33" t="s">
+      <c r="C19" s="58">
+        <v>2</v>
+      </c>
+      <c r="D19" s="58">
+        <v>2</v>
+      </c>
+      <c r="E19" s="58">
+        <v>2</v>
+      </c>
+      <c r="F19" s="58">
+        <v>2</v>
+      </c>
+      <c r="G19" s="58">
+        <v>2</v>
+      </c>
+      <c r="H19" s="56" t="s">
         <v>187</v>
       </c>
-      <c r="C17" s="52">
-        <v>0.2388888888888889</v>
-      </c>
-      <c r="D17" s="56">
-        <v>0.16429278554634325</v>
-      </c>
-      <c r="E17" s="53">
-        <v>0.12103325269620419</v>
-      </c>
-      <c r="F17" s="53">
-        <v>0.10103766643260505</v>
-      </c>
-      <c r="G17" s="53">
-        <v>0.09098580037985765</v>
-      </c>
-      <c r="H17" s="55" t="s">
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="34" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="33" t="s">
-        <v>135</v>
-      </c>
-      <c r="C18" s="52">
-        <v>-0.19583333333333333</v>
-      </c>
-      <c r="D18" s="53">
-        <v>0.12182361918904425</v>
-      </c>
-      <c r="E18" s="53">
-        <v>0.2798374764653877</v>
-      </c>
-      <c r="F18" s="53">
-        <v>0.16516453995508906</v>
-      </c>
-      <c r="G18" s="53">
-        <v>0.12673281379661727</v>
-      </c>
-      <c r="H18" s="55" t="s">
+      <c r="C20" s="59" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="33" t="s">
+      <c r="D20" s="59" t="s">
+        <v>189</v>
+      </c>
+      <c r="E20" s="59" t="s">
+        <v>189</v>
+      </c>
+      <c r="F20" s="59" t="s">
+        <v>189</v>
+      </c>
+      <c r="G20" s="59" t="s">
+        <v>189</v>
+      </c>
+      <c r="H20" s="56" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="C19" s="57">
-        <v>2</v>
-      </c>
-      <c r="D19" s="57">
-        <v>2</v>
-      </c>
-      <c r="E19" s="57">
-        <v>2</v>
-      </c>
-      <c r="F19" s="57">
-        <v>2</v>
-      </c>
-      <c r="G19" s="57">
-        <v>2</v>
-      </c>
-      <c r="H19" s="55" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="33" t="s">
-        <v>192</v>
-      </c>
-      <c r="C20" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="D20" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="E20" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="F20" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="G20" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="H20" s="55" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="33" t="s">
-        <v>194</v>
-      </c>
-      <c r="C21" s="59" t="str">
+      <c r="C21" s="60" t="str">
         <f>IF('5-Year P&amp;L'!C24&gt;=0,"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="D21" s="59" t="str">
+      <c r="D21" s="60" t="str">
         <f>IF(AND('5-Year P&amp;L'!D24&gt;=0,'5-Year P&amp;L'!C24&lt;0),"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="E21" s="40" t="str">
+      <c r="E21" s="41" t="str">
         <f>IF(AND('5-Year P&amp;L'!E24&gt;=0,'5-Year P&amp;L'!D24&lt;0),"✓ Break-even","")</f>
         <v>✓ Break-even</v>
       </c>
-      <c r="F21" s="59" t="str">
+      <c r="F21" s="60" t="str">
         <f>IF(AND('5-Year P&amp;L'!F24&gt;=0,'5-Year P&amp;L'!E24&lt;0),"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="G21" s="59" t="str">
+      <c r="G21" s="60" t="str">
         <f>IF(AND('5-Year P&amp;L'!G24&gt;=0,'5-Year P&amp;L'!F24&lt;0),"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="H21" s="55" t="s">
-        <v>107</v>
+      <c r="H21" s="56" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="C22" s="61">
+        <v>-2</v>
+      </c>
+      <c r="D22" s="61">
+        <v>0</v>
+      </c>
+      <c r="E22" s="61">
+        <v>5</v>
+      </c>
+      <c r="F22" s="61">
+        <v>6</v>
+      </c>
+      <c r="G22" s="61">
+        <v>6</v>
+      </c>
+      <c r="H22" s="56" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" s="51" t="s">
+        <v>194</v>
+      </c>
+      <c r="D24" s="51" t="s">
         <v>195</v>
       </c>
-      <c r="C22" s="60">
-        <v>-2</v>
-      </c>
-      <c r="D22" s="60">
-        <v>0</v>
-      </c>
-      <c r="E22" s="60">
-        <v>5</v>
-      </c>
-      <c r="F22" s="60">
-        <v>6</v>
-      </c>
-      <c r="G22" s="60">
-        <v>6</v>
-      </c>
-      <c r="H22" s="55" t="s">
+      <c r="E24" s="51"/>
+      <c r="F24" s="51" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="24" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="50" t="s">
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
+    </row>
+    <row r="25" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="62" t="s">
         <v>197</v>
       </c>
-      <c r="C24" s="50" t="s">
+      <c r="C25" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="D24" s="50" t="s">
+      <c r="D25" s="64" t="s">
         <v>199</v>
       </c>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50" t="s">
+      <c r="E25" s="64"/>
+      <c r="F25" s="65" t="s">
         <v>200</v>
       </c>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
-    </row>
-    <row r="25" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="61" t="s">
+      <c r="G25" s="65"/>
+      <c r="H25" s="65"/>
+    </row>
+    <row r="26" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="62" t="s">
         <v>201</v>
       </c>
-      <c r="C25" s="62" t="s">
+      <c r="C26" s="66" t="s">
         <v>202</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D26" s="64" t="s">
         <v>203</v>
       </c>
-      <c r="E25" s="63"/>
-      <c r="F25" s="64" t="s">
+      <c r="E26" s="64"/>
+      <c r="F26" s="65" t="s">
         <v>204</v>
       </c>
-      <c r="G25" s="64"/>
-      <c r="H25" s="64"/>
-    </row>
-    <row r="26" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="61" t="s">
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
+    </row>
+    <row r="27" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C26" s="65" t="s">
+      <c r="C27" s="41" t="s">
         <v>206</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="D27" s="64" t="s">
         <v>207</v>
       </c>
-      <c r="E26" s="63"/>
-      <c r="F26" s="64" t="s">
+      <c r="E27" s="64"/>
+      <c r="F27" s="65" t="s">
         <v>208</v>
       </c>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-    </row>
-    <row r="27" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B27" s="61" t="s">
+      <c r="G27" s="65"/>
+      <c r="H27" s="65"/>
+    </row>
+    <row r="28" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="62" t="s">
         <v>209</v>
       </c>
-      <c r="C27" s="40" t="s">
+      <c r="C28" s="41" t="s">
+        <v>206</v>
+      </c>
+      <c r="D28" s="64" t="s">
         <v>210</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="E28" s="64"/>
+      <c r="F28" s="65" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="63"/>
-      <c r="F27" s="64" t="s">
+      <c r="G28" s="65"/>
+      <c r="H28" s="65"/>
+    </row>
+    <row r="29" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="62" t="s">
         <v>212</v>
       </c>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-    </row>
-    <row r="28" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="61" t="s">
+      <c r="C29" s="41" t="s">
+        <v>206</v>
+      </c>
+      <c r="D29" s="64" t="s">
         <v>213</v>
       </c>
-      <c r="C28" s="40" t="s">
-        <v>210</v>
-      </c>
-      <c r="D28" s="63" t="s">
+      <c r="E29" s="64"/>
+      <c r="F29" s="65" t="s">
         <v>214</v>
       </c>
-      <c r="E28" s="63"/>
-      <c r="F28" s="64" t="s">
+      <c r="G29" s="65"/>
+      <c r="H29" s="65"/>
+    </row>
+    <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="G28" s="64"/>
-      <c r="H28" s="64"/>
-    </row>
-    <row r="29" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="61" t="s">
+      <c r="C30" s="41" t="s">
+        <v>206</v>
+      </c>
+      <c r="D30" s="64" t="s">
         <v>216</v>
       </c>
-      <c r="C29" s="40" t="s">
-        <v>210</v>
-      </c>
-      <c r="D29" s="63" t="s">
+      <c r="E30" s="64"/>
+      <c r="F30" s="65" t="s">
         <v>217</v>
       </c>
-      <c r="E29" s="63"/>
-      <c r="F29" s="64" t="s">
+      <c r="G30" s="65"/>
+      <c r="H30" s="65"/>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="62" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="34" t="s">
         <v>218</v>
       </c>
-      <c r="G29" s="64"/>
-      <c r="H29" s="64"/>
-    </row>
-    <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="61" t="s">
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B34" s="67" t="s">
         <v>219</v>
       </c>
-      <c r="C30" s="40" t="s">
-        <v>210</v>
-      </c>
-      <c r="D30" s="63" t="s">
-        <v>220</v>
-      </c>
-      <c r="E30" s="63"/>
-      <c r="F30" s="64" t="s">
-        <v>221</v>
-      </c>
-      <c r="G30" s="64"/>
-      <c r="H30" s="64"/>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="61" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="33" t="s">
-        <v>222</v>
-      </c>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="66" t="s">
-        <v>223</v>
-      </c>
-      <c r="C34" s="66"/>
-      <c r="D34" s="66"/>
-      <c r="E34" s="66"/>
-      <c r="F34" s="66"/>
-      <c r="G34" s="66"/>
-      <c r="H34" s="66"/>
+      <c r="C34" s="67"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="67"/>
+      <c r="F34" s="67"/>
+      <c r="G34" s="67"/>
+      <c r="H34" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -2557,13 +2552,14 @@
     <tabColor rgb="FFD97706"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E72"/>
+  <dimension ref="B1:H72"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
@@ -2965,51 +2961,145 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="66" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B66" s="17" t="s">
         <v>95</v>
       </c>
       <c r="C66" s="17"/>
       <c r="D66" s="17"/>
-    </row>
-    <row r="68" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="E66" s="17"/>
+      <c r="F66" s="17"/>
+      <c r="G66" s="17"/>
+      <c r="H66" s="17"/>
+    </row>
+    <row r="67" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C67" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="D67" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="E67" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="F67" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="G67" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="H67" s="24" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="68" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C68" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D68" s="23" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="69" spans="3:4" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+      <c r="D68" s="20">
+        <v>3</v>
+      </c>
+      <c r="E68" s="20">
+        <v>4</v>
+      </c>
+      <c r="F68" s="20">
+        <v>5</v>
+      </c>
+      <c r="G68" s="20">
+        <v>6</v>
+      </c>
+      <c r="H68" s="20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C69" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="D69" s="23" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="70" spans="3:4" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+      <c r="D69" s="20">
+        <v>2</v>
+      </c>
+      <c r="E69" s="20">
+        <v>3</v>
+      </c>
+      <c r="F69" s="20">
+        <v>4</v>
+      </c>
+      <c r="G69" s="20">
+        <v>5</v>
+      </c>
+      <c r="H69" s="20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C70" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="D70" s="23" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C71" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="D71" s="25" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="72" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C72" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="D72" s="27" t="s">
+      <c r="D70" s="20">
+        <v>5</v>
+      </c>
+      <c r="E70" s="20">
+        <v>7</v>
+      </c>
+      <c r="F70" s="20">
+        <v>9</v>
+      </c>
+      <c r="G70" s="20">
+        <v>10</v>
+      </c>
+      <c r="H70" s="20">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C71" s="25" t="s">
         <v>105</v>
+      </c>
+      <c r="D71" s="26">
+        <f>D68+D69+D70</f>
+        <v>10</v>
+      </c>
+      <c r="E71" s="26">
+        <f>E68+E69+E70</f>
+        <v>14</v>
+      </c>
+      <c r="F71" s="26">
+        <f>F68+F69+F70</f>
+        <v>18</v>
+      </c>
+      <c r="G71" s="26">
+        <f>G68+G69+G70</f>
+        <v>21</v>
+      </c>
+      <c r="H71" s="26">
+        <f>H68+H69+H70</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="72" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C72" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="D72" s="28">
+        <f>IF(D12=0,0,D71/D12)</f>
+        <v>0.66666667</v>
+      </c>
+      <c r="E72" s="28">
+        <f>IF(D13=0,0,E71/D13)</f>
+        <v>0.63636364</v>
+      </c>
+      <c r="F72" s="28">
+        <f>IF(D14=0,0,F71/D14)</f>
+        <v>0.6</v>
+      </c>
+      <c r="G72" s="28">
+        <f>IF(D15=0,0,G71/D15)</f>
+        <v>0.58333333</v>
+      </c>
+      <c r="H72" s="28">
+        <f>IF(D16=0,0,H71/D16)</f>
+        <v>0.575</v>
       </c>
     </row>
   </sheetData>
@@ -3021,7 +3111,7 @@
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B66:H66"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -3047,7 +3137,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3056,444 +3146,444 @@
       <c r="G1" s="13"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="28"/>
-      <c r="C3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="29" t="s">
+      <c r="B3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="E3" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="31">
+      <c r="C4" s="32">
         <f>Assumptions!D12</f>
         <v>15</v>
       </c>
-      <c r="D4" s="31">
+      <c r="D4" s="32">
         <f>Assumptions!D13</f>
         <v>22</v>
       </c>
-      <c r="E4" s="31">
+      <c r="E4" s="32">
         <f>Assumptions!D14</f>
         <v>30</v>
       </c>
-      <c r="F4" s="31">
+      <c r="F4" s="32">
         <f>Assumptions!D15</f>
         <v>36</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="32">
         <f>Assumptions!D16</f>
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="32" t="str">
+      <c r="B5" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="33" t="str">
         <f>Assumptions!D12*Assumptions!D20</f>
         <v>0</v>
       </c>
-      <c r="D5" s="32" t="str">
+      <c r="D5" s="33" t="str">
         <f>Assumptions!D13*Assumptions!D20*(1+Assumptions!D21)^1</f>
         <v>0</v>
       </c>
-      <c r="E5" s="32" t="str">
+      <c r="E5" s="33" t="str">
         <f>Assumptions!D14*Assumptions!D20*(1+Assumptions!D21)^2</f>
         <v>0</v>
       </c>
-      <c r="F5" s="32" t="str">
+      <c r="F5" s="33" t="str">
         <f>Assumptions!D15*Assumptions!D20*(1+Assumptions!D21)^3</f>
         <v>0</v>
       </c>
-      <c r="G5" s="32" t="str">
+      <c r="G5" s="33" t="str">
         <f>Assumptions!D16*Assumptions!D20*(1+Assumptions!D21)^4</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="C6" s="32" t="str">
+      <c r="B6" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="33" t="str">
         <f>C5*Assumptions!D26</f>
         <v>0</v>
       </c>
-      <c r="D6" s="32" t="str">
+      <c r="D6" s="33" t="str">
         <f>D5*Assumptions!D26</f>
         <v>0</v>
       </c>
-      <c r="E6" s="32" t="str">
+      <c r="E6" s="33" t="str">
         <f>E5*Assumptions!D26</f>
         <v>0</v>
       </c>
-      <c r="F6" s="32" t="str">
+      <c r="F6" s="33" t="str">
         <f>F5*Assumptions!D26</f>
         <v>0</v>
       </c>
-      <c r="G6" s="32" t="str">
+      <c r="G6" s="33" t="str">
         <f>G5*Assumptions!D26</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" s="32">
+      <c r="B7" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="33">
         <f>Assumptions!D12*Assumptions!D22</f>
         <v>105000</v>
       </c>
-      <c r="D7" s="32">
+      <c r="D7" s="33">
         <f>Assumptions!D13*Assumptions!D22*(1+Assumptions!D23)^1</f>
         <v>158620</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="33">
         <f>Assumptions!D14*Assumptions!D22*(1+Assumptions!D23)^2</f>
         <v>222789</v>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="33">
         <f>Assumptions!D15*Assumptions!D22*(1+Assumptions!D23)^3</f>
         <v>275367.204</v>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="33">
         <f>Assumptions!D16*Assumptions!D22*(1+Assumptions!D23)^4</f>
         <v>315142.4668</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="32" t="str">
+      <c r="B8" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="33" t="str">
         <f>Assumptions!D12*Assumptions!D24</f>
         <v>0</v>
       </c>
-      <c r="D8" s="32" t="str">
+      <c r="D8" s="33" t="str">
         <f>Assumptions!D13*Assumptions!D24*(1+Assumptions!D25)^1</f>
         <v>0</v>
       </c>
-      <c r="E8" s="32" t="str">
+      <c r="E8" s="33" t="str">
         <f>Assumptions!D14*Assumptions!D24*(1+Assumptions!D25)^2</f>
         <v>0</v>
       </c>
-      <c r="F8" s="32" t="str">
+      <c r="F8" s="33" t="str">
         <f>Assumptions!D15*Assumptions!D24*(1+Assumptions!D25)^3</f>
         <v>0</v>
       </c>
-      <c r="G8" s="32" t="str">
+      <c r="G8" s="33" t="str">
         <f>Assumptions!D16*Assumptions!D24*(1+Assumptions!D25)^4</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="32">
+      <c r="B9" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="33">
         <f>Assumptions!D27</f>
         <v>3000</v>
       </c>
-      <c r="D9" s="32">
+      <c r="D9" s="33">
         <f>Assumptions!D27*(1+Assumptions!D28)^1</f>
         <v>3000</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="33">
         <f>Assumptions!D27*(1+Assumptions!D28)^2</f>
         <v>3000</v>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="33">
         <f>Assumptions!D27*(1+Assumptions!D28)^3</f>
         <v>3000</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="33">
         <f>Assumptions!D27*(1+Assumptions!D28)^4</f>
         <v>3000</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="34">
+      <c r="B10" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="35">
         <f>C6+C7+C8+C9</f>
         <v>108000</v>
       </c>
-      <c r="D10" s="34">
+      <c r="D10" s="35">
         <f>D6+D7+D8+D9</f>
         <v>161620</v>
       </c>
-      <c r="E10" s="34">
+      <c r="E10" s="35">
         <f>E6+E7+E8+E9</f>
         <v>225789</v>
       </c>
-      <c r="F10" s="34">
+      <c r="F10" s="35">
         <f>F6+F7+F8+F9</f>
         <v>278367.204</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="35">
         <f>G6+G7+G8+G9</f>
         <v>318142.4668</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="C12" s="31">
+      <c r="B12" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="32">
         <f>CEILING(Assumptions!D12/Assumptions!D32,1)</f>
         <v>1</v>
       </c>
-      <c r="D12" s="31">
+      <c r="D12" s="32">
         <f>CEILING(Assumptions!D13/Assumptions!D32,1)</f>
         <v>1</v>
       </c>
-      <c r="E12" s="31">
+      <c r="E12" s="32">
         <f>CEILING(Assumptions!D14/Assumptions!D32,1)</f>
         <v>1</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="32">
         <f>CEILING(Assumptions!D15/Assumptions!D32,1)</f>
         <v>2</v>
       </c>
-      <c r="G12" s="31">
+      <c r="G12" s="32">
         <f>CEILING(Assumptions!D16/Assumptions!D32,1)</f>
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="C13" s="32">
+      <c r="B13" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="33">
         <f>C12*Assumptions!D33</f>
         <v>30000</v>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="33">
         <f>D12*Assumptions!D33*(1+Assumptions!D34)^1</f>
         <v>30900</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="33">
         <f>E12*Assumptions!D33*(1+Assumptions!D34)^2</f>
         <v>31827</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="33">
         <f>F12*Assumptions!D33*(1+Assumptions!D34)^3</f>
         <v>65563.62</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="33">
         <f>G12*Assumptions!D33*(1+Assumptions!D34)^4</f>
         <v>67530.5286</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="C14" s="32">
+      <c r="B14" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" s="33">
         <f>Assumptions!D35*Assumptions!D40</f>
         <v>48000</v>
       </c>
-      <c r="D14" s="32">
+      <c r="D14" s="33">
         <f>Assumptions!D36*Assumptions!D40*(1+Assumptions!D41)^1</f>
         <v>49440</v>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="33">
         <f>Assumptions!D37*Assumptions!D40*(1+Assumptions!D41)^2</f>
         <v>50923.2</v>
       </c>
-      <c r="F14" s="32">
+      <c r="F14" s="33">
         <f>Assumptions!D38*Assumptions!D40*(1+Assumptions!D41)^3</f>
         <v>52450.896</v>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="33">
         <f>Assumptions!D39*Assumptions!D40*(1+Assumptions!D41)^4</f>
         <v>54024.42288</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="30" t="s">
-        <v>122</v>
-      </c>
-      <c r="C15" s="32">
+      <c r="B15" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="33">
         <f>(C13+C14)*Assumptions!D42</f>
         <v>15600</v>
       </c>
-      <c r="D15" s="32">
+      <c r="D15" s="33">
         <f>(D13+D14)*Assumptions!D42</f>
         <v>16068</v>
       </c>
-      <c r="E15" s="32">
+      <c r="E15" s="33">
         <f>(E13+E14)*Assumptions!D42</f>
         <v>16550.04</v>
       </c>
-      <c r="F15" s="32">
+      <c r="F15" s="33">
         <f>(F13+F14)*Assumptions!D42</f>
         <v>23602.9032</v>
       </c>
-      <c r="G15" s="32">
+      <c r="G15" s="33">
         <f>(G13+G14)*Assumptions!D42</f>
         <v>24310.990296</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B16" s="33" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="34">
+      <c r="B16" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="35">
         <f>C13+C14+C15</f>
         <v>93600</v>
       </c>
-      <c r="D16" s="34">
+      <c r="D16" s="35">
         <f>D13+D14+D15</f>
         <v>96408</v>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="35">
         <f>E13+E14+E15</f>
         <v>99300.24</v>
       </c>
-      <c r="F16" s="34">
+      <c r="F16" s="35">
         <f>F13+F14+F15</f>
         <v>141617.4192</v>
       </c>
-      <c r="G16" s="34">
+      <c r="G16" s="35">
         <f>G13+G14+G15</f>
         <v>145865.941776</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="C18" s="32">
+      <c r="B18" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="C18" s="33">
         <f>Assumptions!D46</f>
         <v>21600</v>
       </c>
-      <c r="D18" s="32">
+      <c r="D18" s="33">
         <f>Assumptions!D46*(1+Assumptions!D47)^1</f>
         <v>22230.41860465</v>
       </c>
-      <c r="E18" s="32">
+      <c r="E18" s="33">
         <f>Assumptions!D46*(1+Assumptions!D47)^2</f>
         <v>22879.23663602</v>
       </c>
-      <c r="F18" s="32">
+      <c r="F18" s="33">
         <f>Assumptions!D46*(1+Assumptions!D47)^3</f>
         <v>23546.99110063</v>
       </c>
-      <c r="G18" s="32">
+      <c r="G18" s="33">
         <f>Assumptions!D46*(1+Assumptions!D47)^4</f>
         <v>24234.2346781</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="30" t="s">
-        <v>125</v>
-      </c>
-      <c r="C19" s="32">
+      <c r="B19" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="33">
         <f>Assumptions!D48</f>
         <v>4200</v>
       </c>
-      <c r="D19" s="32">
+      <c r="D19" s="33">
         <f>Assumptions!D48*(1+Assumptions!D49)^1</f>
         <v>4322.58139535</v>
       </c>
-      <c r="E19" s="32">
+      <c r="E19" s="33">
         <f>Assumptions!D48*(1+Assumptions!D49)^2</f>
         <v>4448.740457</v>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="33">
         <f>Assumptions!D48*(1+Assumptions!D49)^3</f>
         <v>4578.5816029</v>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="33">
         <f>Assumptions!D48*(1+Assumptions!D49)^4</f>
         <v>4712.21229852</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="C20" s="32">
+      <c r="B20" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="33">
         <f>Assumptions!D12*Assumptions!D50</f>
         <v>6000</v>
       </c>
-      <c r="D20" s="32">
+      <c r="D20" s="33">
         <f>Assumptions!D13*Assumptions!D50*(1+Assumptions!D51)^1</f>
         <v>13293.86666667</v>
       </c>
-      <c r="E20" s="32">
+      <c r="E20" s="33">
         <f>Assumptions!D14*Assumptions!D50*(1+Assumptions!D51)^2</f>
         <v>27385.36533333</v>
       </c>
-      <c r="F20" s="32">
+      <c r="F20" s="33">
         <f>Assumptions!D15*Assumptions!D50*(1+Assumptions!D51)^3</f>
         <v>49644.19027627</v>
       </c>
-      <c r="G20" s="32">
+      <c r="G20" s="33">
         <f>Assumptions!D16*Assumptions!D50*(1+Assumptions!D51)^4</f>
         <v>83328.69271557</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="C21" s="32">
+      <c r="B21" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="33">
         <f>Assumptions!D52</f>
         <v>3750</v>
       </c>
-      <c r="D21" s="32">
+      <c r="D21" s="33">
         <f>Assumptions!D52*(1+Assumptions!D53)^1</f>
         <v>5676</v>
       </c>
-      <c r="E21" s="32">
+      <c r="E21" s="33">
         <f>Assumptions!D52*(1+Assumptions!D53)^2</f>
         <v>8591.1936</v>
       </c>
-      <c r="F21" s="32">
+      <c r="F21" s="33">
         <f>Assumptions!D52*(1+Assumptions!D53)^3</f>
         <v>13003.63063296</v>
       </c>
-      <c r="G21" s="32">
+      <c r="G21" s="33">
         <f>Assumptions!D52*(1+Assumptions!D53)^4</f>
         <v>19682.29532605</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="33" t="s">
-        <v>128</v>
-      </c>
-      <c r="C22" s="34">
+      <c r="B22" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="35">
         <f>C18+C19+C20+C21</f>
         <v>35550</v>
       </c>
-      <c r="D22" s="34">
+      <c r="D22" s="35">
         <f>D18+D19+D20+D21</f>
         <v>45522.86666667</v>
       </c>
-      <c r="E22" s="34">
+      <c r="E22" s="35">
         <f>E18+E19+E20+E21</f>
         <v>63304.53602636</v>
       </c>
-      <c r="F22" s="34">
+      <c r="F22" s="35">
         <f>F18+F19+F20+F21</f>
         <v>90773.39361276</v>
       </c>
-      <c r="G22" s="34">
+      <c r="G22" s="35">
         <f>G18+G19+G20+G21</f>
         <v>131957.43501824</v>
       </c>
@@ -3526,7 +3616,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3535,415 +3625,415 @@
       <c r="G1" s="13"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="28"/>
-      <c r="C3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="29" t="s">
+      <c r="B3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="E3" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="C5" s="31">
+      <c r="C5" s="32">
         <f>Drivers!C4</f>
         <v>15</v>
       </c>
-      <c r="D5" s="31">
+      <c r="D5" s="32">
         <f>Drivers!D4</f>
         <v>22</v>
       </c>
-      <c r="E5" s="31">
+      <c r="E5" s="32">
         <f>Drivers!E4</f>
         <v>30</v>
       </c>
-      <c r="F5" s="31">
+      <c r="F5" s="32">
         <f>Drivers!F4</f>
         <v>36</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="32">
         <f>Drivers!G4</f>
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="C6" s="32" t="str">
+      <c r="B6" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="33" t="str">
         <f>Drivers!C6</f>
         <v>0</v>
       </c>
-      <c r="D6" s="32" t="str">
+      <c r="D6" s="33" t="str">
         <f>Drivers!D6</f>
         <v>0</v>
       </c>
-      <c r="E6" s="32" t="str">
+      <c r="E6" s="33" t="str">
         <f>Drivers!E6</f>
         <v>0</v>
       </c>
-      <c r="F6" s="32" t="str">
+      <c r="F6" s="33" t="str">
         <f>Drivers!F6</f>
         <v>0</v>
       </c>
-      <c r="G6" s="32" t="str">
+      <c r="G6" s="33" t="str">
         <f>Drivers!G6</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
-        <v>130</v>
-      </c>
-      <c r="C7" s="32">
+      <c r="B7" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="33">
         <f>Drivers!C7</f>
         <v>105000</v>
       </c>
-      <c r="D7" s="32">
+      <c r="D7" s="33">
         <f>Drivers!D7</f>
         <v>158620</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="33">
         <f>Drivers!E7</f>
         <v>222789</v>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="33">
         <f>Drivers!F7</f>
         <v>275367.204</v>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="33">
         <f>Drivers!G7</f>
         <v>315142.4668</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
-        <v>131</v>
-      </c>
-      <c r="C8" s="32" t="str">
+      <c r="B8" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="33" t="str">
         <f>Drivers!C8</f>
         <v>0</v>
       </c>
-      <c r="D8" s="32" t="str">
+      <c r="D8" s="33" t="str">
         <f>Drivers!D8</f>
         <v>0</v>
       </c>
-      <c r="E8" s="32" t="str">
+      <c r="E8" s="33" t="str">
         <f>Drivers!E8</f>
         <v>0</v>
       </c>
-      <c r="F8" s="32" t="str">
+      <c r="F8" s="33" t="str">
         <f>Drivers!F8</f>
         <v>0</v>
       </c>
-      <c r="G8" s="32" t="str">
+      <c r="G8" s="33" t="str">
         <f>Drivers!G8</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="32">
+      <c r="B9" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="33">
         <f>Drivers!C9</f>
         <v>3000</v>
       </c>
-      <c r="D9" s="32">
+      <c r="D9" s="33">
         <f>Drivers!D9</f>
         <v>3000</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="33">
         <f>Drivers!E9</f>
         <v>3000</v>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="33">
         <f>Drivers!F9</f>
         <v>3000</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="33">
         <f>Drivers!G9</f>
         <v>3000</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="34">
+      <c r="B10" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="35">
         <f>Drivers!C10</f>
         <v>108000</v>
       </c>
-      <c r="D10" s="34">
+      <c r="D10" s="35">
         <f>Drivers!D10</f>
         <v>161620</v>
       </c>
-      <c r="E10" s="34">
+      <c r="E10" s="35">
         <f>Drivers!E10</f>
         <v>225789</v>
       </c>
-      <c r="F10" s="34">
+      <c r="F10" s="35">
         <f>Drivers!F10</f>
         <v>278367.204</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="35">
         <f>Drivers!G10</f>
         <v>318142.4668</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="C12" s="32">
+      <c r="B12" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="33">
         <f>Drivers!C16</f>
         <v>93600</v>
       </c>
-      <c r="D12" s="32">
+      <c r="D12" s="33">
         <f>Drivers!D16</f>
         <v>96408</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="33">
         <f>Drivers!E16</f>
         <v>99300.24</v>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="33">
         <f>Drivers!F16</f>
         <v>141617.4192</v>
       </c>
-      <c r="G12" s="32">
+      <c r="G12" s="33">
         <f>Drivers!G16</f>
         <v>145865.941776</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="32">
+      <c r="B13" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="33">
         <f>Drivers!C22</f>
         <v>35550</v>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="33">
         <f>Drivers!D22</f>
         <v>45522.86666667</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="33">
         <f>Drivers!E22</f>
         <v>63304.53602636</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="33">
         <f>Drivers!F22</f>
         <v>90773.39361276</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="33">
         <f>Drivers!G22</f>
         <v>131957.43501824</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="33" t="s">
-        <v>133</v>
-      </c>
-      <c r="C15" s="34">
+      <c r="B15" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="C15" s="35">
         <f>C12+C13</f>
         <v>129150</v>
       </c>
-      <c r="D15" s="34">
+      <c r="D15" s="35">
         <f>D12+D13</f>
         <v>141930.86666667</v>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="35">
         <f>E12+E13</f>
         <v>162604.77602636</v>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="35">
         <f>F12+F13</f>
         <v>232390.81281276</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="35">
         <f>G12+G13</f>
         <v>277823.37679424</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B16" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="C16" s="35">
+      <c r="B16" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="36">
         <f>C10-C15</f>
         <v>-21150</v>
       </c>
-      <c r="D16" s="36">
+      <c r="D16" s="37">
         <f>D10-D15</f>
         <v>19689.13333333</v>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="37">
         <f>E10-E15</f>
         <v>63184.22397364</v>
       </c>
-      <c r="F16" s="36">
+      <c r="F16" s="37">
         <f>F10-F15</f>
         <v>45976.39118724</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="37">
         <f>G10-G15</f>
         <v>40319.09000576</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="C17" s="37">
+      <c r="B17" s="31" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="38">
         <f>IF(C10&gt;0,C16/C10,0)</f>
         <v>-0.19583333</v>
       </c>
-      <c r="D17" s="37">
+      <c r="D17" s="38">
         <f>IF(D10&gt;0,D16/D10,0)</f>
         <v>0.12182362</v>
       </c>
-      <c r="E17" s="37">
+      <c r="E17" s="38">
         <f>IF(E10&gt;0,E16/E10,0)</f>
         <v>0.27983748</v>
       </c>
-      <c r="F17" s="37">
+      <c r="F17" s="38">
         <f>IF(F10&gt;0,F16/F10,0)</f>
         <v>0.16516454</v>
       </c>
-      <c r="G17" s="37">
+      <c r="G17" s="38">
         <f>IF(G10&gt;0,G16/G10,0)</f>
         <v>0.12673281</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="C19" s="32" t="str">
+      <c r="B19" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="C19" s="33" t="str">
         <f>'Cash Flow &amp; DSCR'!C9</f>
         <v>0</v>
       </c>
-      <c r="D19" s="32" t="str">
+      <c r="D19" s="33" t="str">
         <f>'Cash Flow &amp; DSCR'!D9</f>
         <v>0</v>
       </c>
-      <c r="E19" s="32" t="str">
+      <c r="E19" s="33" t="str">
         <f>'Cash Flow &amp; DSCR'!E9</f>
         <v>0</v>
       </c>
-      <c r="F19" s="32" t="str">
+      <c r="F19" s="33" t="str">
         <f>'Cash Flow &amp; DSCR'!F9</f>
         <v>0</v>
       </c>
-      <c r="G19" s="32" t="str">
+      <c r="G19" s="33" t="str">
         <f>'Cash Flow &amp; DSCR'!G9</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="33" t="s">
-        <v>137</v>
-      </c>
-      <c r="C21" s="35">
+      <c r="B21" s="34" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" s="36">
         <f>C16-C19</f>
         <v>-21150</v>
       </c>
-      <c r="D21" s="36">
+      <c r="D21" s="37">
         <f>D16-D19</f>
         <v>19689.13333333</v>
       </c>
-      <c r="E21" s="36">
+      <c r="E21" s="37">
         <f>E16-E19</f>
         <v>63184.22397364</v>
       </c>
-      <c r="F21" s="36">
+      <c r="F21" s="37">
         <f>F16-F19</f>
         <v>45976.39118724</v>
       </c>
-      <c r="G21" s="36">
+      <c r="G21" s="37">
         <f>G16-G19</f>
         <v>40319.09000576</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="30" t="s">
-        <v>138</v>
-      </c>
-      <c r="C22" s="37">
+      <c r="B22" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" s="38">
         <f>IF(C10&gt;0,C21/C10,0)</f>
         <v>-0.19583333</v>
       </c>
-      <c r="D22" s="37">
+      <c r="D22" s="38">
         <f>IF(D10&gt;0,D21/D10,0)</f>
         <v>0.12182362</v>
       </c>
-      <c r="E22" s="37">
+      <c r="E22" s="38">
         <f>IF(E10&gt;0,E21/E10,0)</f>
         <v>0.27983748</v>
       </c>
-      <c r="F22" s="37">
+      <c r="F22" s="38">
         <f>IF(F10&gt;0,F21/F10,0)</f>
         <v>0.16516454</v>
       </c>
-      <c r="G22" s="37">
+      <c r="G22" s="38">
         <f>IF(G10&gt;0,G21/G10,0)</f>
         <v>0.12673281</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B24" s="33" t="s">
-        <v>139</v>
-      </c>
-      <c r="C24" s="38">
+      <c r="B24" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="C24" s="39">
         <f>C21</f>
         <v>-21150</v>
       </c>
-      <c r="D24" s="38">
+      <c r="D24" s="39">
         <f>C24+D21</f>
         <v>-1460.86666667</v>
       </c>
-      <c r="E24" s="38">
+      <c r="E24" s="39">
         <f>D24+E21</f>
         <v>61723.35730698</v>
       </c>
-      <c r="F24" s="38">
+      <c r="F24" s="39">
         <f>E24+F21</f>
         <v>107699.74849422</v>
       </c>
-      <c r="G24" s="38">
+      <c r="G24" s="39">
         <f>F24+G21</f>
         <v>148018.83849998</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B25" s="33" t="s">
-        <v>140</v>
-      </c>
-      <c r="C25" s="39" t="s">
+      <c r="B25" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="D25" s="39" t="s">
+      <c r="D25" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="E25" s="40" t="s">
-        <v>141</v>
-      </c>
-      <c r="F25" s="39" t="s">
+      <c r="E25" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="F25" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="G25" s="39" t="s">
+      <c r="G25" s="40" t="s">
         <v>7</v>
       </c>
     </row>
@@ -3975,7 +4065,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3984,244 +4074,244 @@
       <c r="G1" s="13"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="28"/>
-      <c r="C3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="E3" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>111</v>
+      <c r="B3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="33" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4" s="38" t="str">
+      <c r="B4" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="C4" s="39" t="str">
         <f>Assumptions!D57</f>
         <v>0</v>
       </c>
-      <c r="D4" s="38">
+      <c r="D4" s="39">
         <f>C16</f>
         <v>-21150</v>
       </c>
-      <c r="E4" s="38">
+      <c r="E4" s="39">
         <f>D16</f>
         <v>-1460.86666667</v>
       </c>
-      <c r="F4" s="38">
+      <c r="F4" s="39">
         <f>E16</f>
         <v>61723.35730698</v>
       </c>
-      <c r="G4" s="38">
+      <c r="G4" s="39">
         <f>F16</f>
         <v>107699.74849422</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="32">
+      <c r="B5" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="33">
         <f>'5-Year P&amp;L'!C16</f>
         <v>-21150</v>
       </c>
-      <c r="D5" s="32">
+      <c r="D5" s="33">
         <f>'5-Year P&amp;L'!D16</f>
         <v>19689.13333333</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="33">
         <f>'5-Year P&amp;L'!E16</f>
         <v>63184.22397364</v>
       </c>
-      <c r="F5" s="32">
+      <c r="F5" s="33">
         <f>'5-Year P&amp;L'!F16</f>
         <v>45976.39118724</v>
       </c>
-      <c r="G5" s="32">
+      <c r="G5" s="33">
         <f>'5-Year P&amp;L'!G16</f>
         <v>40319.09000576</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="C7" s="32" t="str">
+      <c r="B7" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="33" t="str">
         <f>Assumptions!D58</f>
         <v>0</v>
       </c>
-      <c r="D7" s="32" t="str">
+      <c r="D7" s="33" t="str">
         <f>Assumptions!D58</f>
         <v>0</v>
       </c>
-      <c r="E7" s="32" t="str">
+      <c r="E7" s="33" t="str">
         <f>Assumptions!D58</f>
         <v>0</v>
       </c>
-      <c r="F7" s="32" t="str">
+      <c r="F7" s="33" t="str">
         <f>Assumptions!D58</f>
         <v>0</v>
       </c>
-      <c r="G7" s="32" t="str">
+      <c r="G7" s="33" t="str">
         <f>Assumptions!D58</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" s="32" t="str">
+      <c r="B8" s="31" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" s="33" t="str">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="32" t="str">
+      <c r="D8" s="33" t="str">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="32" t="str">
+      <c r="E8" s="33" t="str">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="32" t="str">
+      <c r="F8" s="33" t="str">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="32" t="str">
+      <c r="G8" s="33" t="str">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="33" t="s">
-        <v>147</v>
-      </c>
-      <c r="C9" s="34" t="str">
+      <c r="B9" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9" s="35" t="str">
         <f>C7+C8</f>
         <v>0</v>
       </c>
-      <c r="D9" s="34" t="str">
+      <c r="D9" s="35" t="str">
         <f>D7+D8</f>
         <v>0</v>
       </c>
-      <c r="E9" s="34" t="str">
+      <c r="E9" s="35" t="str">
         <f>E7+E8</f>
         <v>0</v>
       </c>
-      <c r="F9" s="34" t="str">
+      <c r="F9" s="35" t="str">
         <f>F7+F8</f>
         <v>0</v>
       </c>
-      <c r="G9" s="34" t="str">
+      <c r="G9" s="35" t="str">
         <f>G7+G8</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="33" t="s">
-        <v>148</v>
-      </c>
-      <c r="C11" s="41" t="str">
+      <c r="B11" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="42" t="str">
         <f>IF(C9&gt;0,C5/C9,IF(C5&gt;0,99.9,0))</f>
         <v>0</v>
       </c>
-      <c r="D11" s="42">
+      <c r="D11" s="43">
         <f>IF(D9&gt;0,D5/D9,IF(D5&gt;0,99.9,0))</f>
         <v>99.9</v>
       </c>
-      <c r="E11" s="42">
+      <c r="E11" s="43">
         <f>IF(E9&gt;0,E5/E9,IF(E5&gt;0,99.9,0))</f>
         <v>99.9</v>
       </c>
-      <c r="F11" s="42">
+      <c r="F11" s="43">
         <f>IF(F9&gt;0,F5/F9,IF(F5&gt;0,99.9,0))</f>
         <v>99.9</v>
       </c>
-      <c r="G11" s="42">
+      <c r="G11" s="43">
         <f>IF(G9&gt;0,G5/G9,IF(G5&gt;0,99.9,0))</f>
         <v>99.9</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="C13" s="32">
+      <c r="B13" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="33">
         <f>C5-C9</f>
         <v>-21150</v>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="33">
         <f>D5-D9</f>
         <v>19689.13333333</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="33">
         <f>E5-E9</f>
         <v>63184.22397364</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="33">
         <f>F5-F9</f>
         <v>45976.39118724</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="33">
         <f>G5-G9</f>
         <v>40319.09000576</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="C14" s="38">
+      <c r="B14" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="C14" s="39">
         <f>C5-C9</f>
         <v>-21150</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="39">
         <f>D5-D9</f>
         <v>19689.13333333</v>
       </c>
-      <c r="E14" s="38">
+      <c r="E14" s="39">
         <f>E5-E9</f>
         <v>63184.22397364</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="39">
         <f>F5-F9</f>
         <v>45976.39118724</v>
       </c>
-      <c r="G14" s="38">
+      <c r="G14" s="39">
         <f>G5-G9</f>
         <v>40319.09000576</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B16" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="C16" s="35">
+      <c r="B16" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" s="36">
         <f>C4+C14</f>
         <v>-21150</v>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="36">
         <f>D4+D14</f>
         <v>-1460.86666667</v>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="37">
         <f>E4+E14</f>
         <v>61723.35730698</v>
       </c>
-      <c r="F16" s="36">
+      <c r="F16" s="37">
         <f>F4+F14</f>
         <v>107699.74849422</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="37">
         <f>G4+G14</f>
         <v>148018.83849998</v>
       </c>
@@ -4254,7 +4344,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -4263,94 +4353,94 @@
       <c r="G1" s="13"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="28"/>
-      <c r="C3" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="E3" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>111</v>
+      <c r="B3" s="29"/>
+      <c r="C3" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="C4" s="31">
+      <c r="B4" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C4" s="32">
         <f>Drivers!C12</f>
         <v>1</v>
       </c>
-      <c r="D4" s="31">
+      <c r="D4" s="32">
         <f>Drivers!D12</f>
         <v>1</v>
       </c>
-      <c r="E4" s="31">
+      <c r="E4" s="32">
         <f>Drivers!E12</f>
         <v>1</v>
       </c>
-      <c r="F4" s="31">
+      <c r="F4" s="32">
         <f>Drivers!F12</f>
         <v>2</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="32">
         <f>Drivers!G12</f>
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="C5" s="31">
+      <c r="B5" s="31" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="32">
         <f>Assumptions!D35</f>
         <v>1</v>
       </c>
-      <c r="D5" s="31">
+      <c r="D5" s="32">
         <f>Assumptions!D36</f>
         <v>1</v>
       </c>
-      <c r="E5" s="31">
+      <c r="E5" s="32">
         <f>Assumptions!D37</f>
         <v>1</v>
       </c>
-      <c r="F5" s="31">
+      <c r="F5" s="32">
         <f>Assumptions!D38</f>
         <v>1</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="32">
         <f>Assumptions!D39</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="33" t="s">
-        <v>155</v>
-      </c>
-      <c r="C6" s="43">
+      <c r="B6" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" s="44">
         <f>C4+C5</f>
         <v>2</v>
       </c>
-      <c r="D6" s="43">
+      <c r="D6" s="44">
         <f>D4+D5</f>
         <v>2</v>
       </c>
-      <c r="E6" s="43">
+      <c r="E6" s="44">
         <f>E4+E5</f>
         <v>2</v>
       </c>
-      <c r="F6" s="43">
+      <c r="F6" s="44">
         <f>F4+F5</f>
         <v>3</v>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="44">
         <f>G4+G5</f>
         <v>3</v>
       </c>
@@ -4383,51 +4473,51 @@
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C1" s="13"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="32" t="str">
+      <c r="B3" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="33" t="str">
         <f>Assumptions!D59</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="C4" s="37">
+      <c r="B4" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" s="38">
         <f>Assumptions!D60</f>
         <v>0.08</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="32">
         <f>Assumptions!D61</f>
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="C6" s="38" t="str">
+      <c r="B6" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C6" s="39" t="str">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="41" t="str">
+      <c r="B8" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="42" t="str">
         <f>'Cash Flow &amp; DSCR'!C11</f>
         <v>0</v>
       </c>
@@ -4460,136 +4550,136 @@
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C1" s="13"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="30" t="str">
+      <c r="C3" s="31" t="str">
         <f>Assumptions!D5</f>
         <v>Liberty Learning Co-Op</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="30" t="str">
+      <c r="C4" s="31" t="str">
         <f>Assumptions!D7</f>
         <v>Homeschool Co-Op</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="30" t="str">
+      <c r="C5" s="31" t="str">
         <f>Assumptions!D6</f>
         <v>AZ</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="C6" s="30">
+      <c r="B6" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="31">
         <f>Assumptions!D8</f>
         <v>2026</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="32">
         <f>Assumptions!D16</f>
         <v>40</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="C9" s="32">
+      <c r="B9" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="C9" s="33">
         <f>Drivers!G10</f>
         <v>318142.4668</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="C10" s="44">
+      <c r="B10" s="31" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="45">
         <f>'5-Year P&amp;L'!G16</f>
         <v>40319.09000576</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="45" t="s">
-        <v>165</v>
-      </c>
-      <c r="C12" s="28"/>
+      <c r="B12" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="C12" s="29"/>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="C13" s="46">
+      <c r="B13" s="31" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" s="47">
         <f>IF(Drivers!G10&gt;0,'5-Year P&amp;L'!G21/Drivers!G10,0)</f>
         <v>0.12673281</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="30" t="s">
-        <v>167</v>
-      </c>
-      <c r="C14" s="37">
+      <c r="B14" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="C14" s="38">
         <f>IF(Drivers!G10&gt;0,Drivers!G16/Drivers!G10,0)</f>
         <v>0.45849252</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="30" t="s">
-        <v>168</v>
-      </c>
-      <c r="C15" s="32">
+      <c r="B15" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="C15" s="33">
         <f>IF(Assumptions!D16&gt;0,Drivers!G10/Assumptions!D16,0)</f>
         <v>7954</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="30" t="s">
-        <v>169</v>
-      </c>
-      <c r="C16" s="32">
+      <c r="B16" s="31" t="s">
+        <v>165</v>
+      </c>
+      <c r="C16" s="33">
         <f>IF(Assumptions!D16&gt;0,('5-Year P&amp;L'!G12+'5-Year P&amp;L'!G13)/Assumptions!D16,0)</f>
         <v>6946</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="C17" s="41" t="str">
+      <c r="B17" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="C17" s="42" t="str">
         <f>'Cash Flow &amp; DSCR'!C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="30" t="s">
-        <v>171</v>
-      </c>
-      <c r="C18" s="42">
+      <c r="B18" s="31" t="s">
+        <v>167</v>
+      </c>
+      <c r="C18" s="43">
         <f>'Cash Flow &amp; DSCR'!G11</f>
         <v>99.9</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C20" s="12"/>
     </row>

</xml_diff>